<commit_message>
vitorias de escocia e australia
</commit_message>
<xml_diff>
--- a/gabarito/Bolao_Copa2026_TurimMFO_Master.xlsx
+++ b/gabarito/Bolao_Copa2026_TurimMFO_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro\projetos\bolão_copa\gabarito\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A06A87A-2EC0-4702-87B2-05DEFBAD04F8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{042B0E6B-764A-4FBC-A78A-D26B91125285}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2340" yWindow="3000" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4976,67 +4976,73 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="29" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="26" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="27" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="28" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="27" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="48" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="47" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="46" fillId="41" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="47" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="51" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="43" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="49" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="48" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="52" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="46" fillId="42" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="49" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="50" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="45" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="46" fillId="43" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="46" fillId="44" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5045,22 +5051,13 @@
     <xf numFmtId="164" fontId="46" fillId="46" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="51" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="52" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="50" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="46" fillId="45" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="50" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="49" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5076,6 +5073,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="24" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5836,7 +5836,7 @@
       <c r="BM1" s="253"/>
     </row>
     <row r="2" spans="1:65" ht="19.95" customHeight="1">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="261" t="s">
         <v>1028</v>
       </c>
       <c r="B2" s="253"/>
@@ -5972,67 +5972,67 @@
         <v>994</v>
       </c>
       <c r="AG3" s="253"/>
-      <c r="AH3" s="273" t="s">
+      <c r="AH3" s="270" t="s">
         <v>996</v>
       </c>
       <c r="AI3" s="253"/>
-      <c r="AJ3" s="273" t="s">
+      <c r="AJ3" s="270" t="s">
         <v>998</v>
       </c>
       <c r="AK3" s="253"/>
-      <c r="AL3" s="273" t="s">
+      <c r="AL3" s="270" t="s">
         <v>1000</v>
       </c>
       <c r="AM3" s="253"/>
-      <c r="AN3" s="273" t="s">
+      <c r="AN3" s="270" t="s">
         <v>1002</v>
       </c>
       <c r="AO3" s="253"/>
-      <c r="AP3" s="273" t="s">
+      <c r="AP3" s="270" t="s">
         <v>1004</v>
       </c>
       <c r="AQ3" s="253"/>
-      <c r="AR3" s="273" t="s">
+      <c r="AR3" s="270" t="s">
         <v>1006</v>
       </c>
       <c r="AS3" s="253"/>
-      <c r="AT3" s="273" t="s">
+      <c r="AT3" s="270" t="s">
         <v>1008</v>
       </c>
       <c r="AU3" s="253"/>
-      <c r="AV3" s="273" t="s">
+      <c r="AV3" s="270" t="s">
         <v>1010</v>
       </c>
       <c r="AW3" s="253"/>
-      <c r="AX3" s="275" t="s">
+      <c r="AX3" s="274" t="s">
         <v>1012</v>
       </c>
       <c r="AY3" s="253"/>
-      <c r="AZ3" s="275" t="s">
+      <c r="AZ3" s="274" t="s">
         <v>1014</v>
       </c>
       <c r="BA3" s="253"/>
-      <c r="BB3" s="275" t="s">
+      <c r="BB3" s="274" t="s">
         <v>1016</v>
       </c>
       <c r="BC3" s="253"/>
-      <c r="BD3" s="275" t="s">
+      <c r="BD3" s="274" t="s">
         <v>1018</v>
       </c>
       <c r="BE3" s="253"/>
-      <c r="BF3" s="281" t="s">
+      <c r="BF3" s="277" t="s">
         <v>1020</v>
       </c>
       <c r="BG3" s="253"/>
-      <c r="BH3" s="281" t="s">
+      <c r="BH3" s="277" t="s">
         <v>1022</v>
       </c>
       <c r="BI3" s="253"/>
-      <c r="BJ3" s="279" t="s">
+      <c r="BJ3" s="273" t="s">
         <v>1024</v>
       </c>
       <c r="BK3" s="253"/>
-      <c r="BL3" s="280" t="s">
+      <c r="BL3" s="275" t="s">
         <v>1026</v>
       </c>
       <c r="BM3" s="253"/>
@@ -6041,131 +6041,131 @@
       <c r="A4" s="210" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="270">
+      <c r="B4" s="272">
         <v>46201</v>
       </c>
       <c r="C4" s="253"/>
-      <c r="D4" s="270">
+      <c r="D4" s="272">
         <v>46202</v>
       </c>
       <c r="E4" s="253"/>
-      <c r="F4" s="270">
+      <c r="F4" s="272">
         <v>46202</v>
       </c>
       <c r="G4" s="253"/>
-      <c r="H4" s="270">
+      <c r="H4" s="272">
         <v>46202</v>
       </c>
       <c r="I4" s="253"/>
-      <c r="J4" s="270">
+      <c r="J4" s="272">
         <v>46203</v>
       </c>
       <c r="K4" s="253"/>
-      <c r="L4" s="270">
+      <c r="L4" s="272">
         <v>46203</v>
       </c>
       <c r="M4" s="253"/>
-      <c r="N4" s="270">
+      <c r="N4" s="272">
         <v>46203</v>
       </c>
       <c r="O4" s="253"/>
-      <c r="P4" s="270">
+      <c r="P4" s="272">
         <v>46204</v>
       </c>
       <c r="Q4" s="253"/>
-      <c r="R4" s="270">
+      <c r="R4" s="272">
         <v>46204</v>
       </c>
       <c r="S4" s="253"/>
-      <c r="T4" s="270">
+      <c r="T4" s="272">
         <v>46204</v>
       </c>
       <c r="U4" s="253"/>
-      <c r="V4" s="270">
+      <c r="V4" s="272">
         <v>46205</v>
       </c>
       <c r="W4" s="253"/>
-      <c r="X4" s="270">
+      <c r="X4" s="272">
         <v>46205</v>
       </c>
       <c r="Y4" s="253"/>
-      <c r="Z4" s="270">
+      <c r="Z4" s="272">
         <v>46205</v>
       </c>
       <c r="AA4" s="253"/>
-      <c r="AB4" s="270">
+      <c r="AB4" s="272">
         <v>46206</v>
       </c>
       <c r="AC4" s="253"/>
-      <c r="AD4" s="270">
+      <c r="AD4" s="272">
         <v>46206</v>
       </c>
       <c r="AE4" s="253"/>
-      <c r="AF4" s="270">
+      <c r="AF4" s="272">
         <v>46206</v>
       </c>
       <c r="AG4" s="253"/>
-      <c r="AH4" s="274">
+      <c r="AH4" s="276">
         <v>46207</v>
       </c>
       <c r="AI4" s="253"/>
-      <c r="AJ4" s="274">
+      <c r="AJ4" s="276">
         <v>46207</v>
       </c>
       <c r="AK4" s="253"/>
-      <c r="AL4" s="274">
+      <c r="AL4" s="276">
         <v>46208</v>
       </c>
       <c r="AM4" s="253"/>
-      <c r="AN4" s="274">
+      <c r="AN4" s="276">
         <v>46208</v>
       </c>
       <c r="AO4" s="253"/>
-      <c r="AP4" s="274">
+      <c r="AP4" s="276">
         <v>46209</v>
       </c>
       <c r="AQ4" s="253"/>
-      <c r="AR4" s="274">
+      <c r="AR4" s="276">
         <v>46209</v>
       </c>
       <c r="AS4" s="253"/>
-      <c r="AT4" s="274">
+      <c r="AT4" s="276">
         <v>46210</v>
       </c>
       <c r="AU4" s="253"/>
-      <c r="AV4" s="274">
+      <c r="AV4" s="276">
         <v>46210</v>
       </c>
       <c r="AW4" s="253"/>
-      <c r="AX4" s="272">
+      <c r="AX4" s="278">
         <v>46212</v>
       </c>
       <c r="AY4" s="253"/>
-      <c r="AZ4" s="272">
+      <c r="AZ4" s="278">
         <v>46213</v>
       </c>
       <c r="BA4" s="253"/>
-      <c r="BB4" s="272">
+      <c r="BB4" s="278">
         <v>46214</v>
       </c>
       <c r="BC4" s="253"/>
-      <c r="BD4" s="272">
+      <c r="BD4" s="278">
         <v>46214</v>
       </c>
       <c r="BE4" s="253"/>
-      <c r="BF4" s="277">
+      <c r="BF4" s="279">
         <v>46217</v>
       </c>
       <c r="BG4" s="253"/>
-      <c r="BH4" s="277">
+      <c r="BH4" s="279">
         <v>46218</v>
       </c>
       <c r="BI4" s="253"/>
-      <c r="BJ4" s="276">
+      <c r="BJ4" s="281">
         <v>46221</v>
       </c>
       <c r="BK4" s="253"/>
-      <c r="BL4" s="278">
+      <c r="BL4" s="280">
         <v>46222</v>
       </c>
       <c r="BM4" s="253"/>
@@ -7620,6 +7620,56 @@
     </row>
   </sheetData>
   <mergeCells count="66">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="AF3:AG3"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="AX4:AY4"/>
+    <mergeCell ref="AH3:AI3"/>
+    <mergeCell ref="AN3:AO3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="AR4:AS4"/>
+    <mergeCell ref="AV4:AW4"/>
+    <mergeCell ref="Z3:AA3"/>
+    <mergeCell ref="AX3:AY3"/>
+    <mergeCell ref="X3:Y3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="AP3:AQ3"/>
+    <mergeCell ref="BB3:BC3"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="R4:S4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="T4:U4"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="AT3:AU3"/>
+    <mergeCell ref="BD3:BE3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="AV3:AW3"/>
+    <mergeCell ref="AD3:AE3"/>
+    <mergeCell ref="BH4:BI4"/>
+    <mergeCell ref="AF4:AG4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AP4:AQ4"/>
+    <mergeCell ref="A1:BM1"/>
+    <mergeCell ref="AT4:AU4"/>
+    <mergeCell ref="AZ4:BA4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="BB4:BC4"/>
+    <mergeCell ref="AJ3:AK3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="BD4:BE4"/>
+    <mergeCell ref="AL3:AM3"/>
+    <mergeCell ref="BF4:BG4"/>
+    <mergeCell ref="BL4:BM4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="X4:Y4"/>
     <mergeCell ref="A2:BM2"/>
     <mergeCell ref="AR3:AS3"/>
     <mergeCell ref="T3:U3"/>
@@ -7636,56 +7686,6 @@
     <mergeCell ref="BF3:BG3"/>
     <mergeCell ref="BH3:BI3"/>
     <mergeCell ref="V4:W4"/>
-    <mergeCell ref="A1:BM1"/>
-    <mergeCell ref="AT4:AU4"/>
-    <mergeCell ref="AZ4:BA4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="BB4:BC4"/>
-    <mergeCell ref="AJ3:AK3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="BD4:BE4"/>
-    <mergeCell ref="AL3:AM3"/>
-    <mergeCell ref="BF4:BG4"/>
-    <mergeCell ref="BL4:BM4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="X4:Y4"/>
-    <mergeCell ref="BH4:BI4"/>
-    <mergeCell ref="AF4:AG4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AP4:AQ4"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="AP3:AQ3"/>
-    <mergeCell ref="BB3:BC3"/>
-    <mergeCell ref="BJ4:BK4"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="R4:S4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="T4:U4"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="AT3:AU3"/>
-    <mergeCell ref="BD3:BE3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="AV3:AW3"/>
-    <mergeCell ref="AD3:AE3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="AF3:AG3"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="AX4:AY4"/>
-    <mergeCell ref="AH3:AI3"/>
-    <mergeCell ref="AN3:AO3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="AR4:AS4"/>
-    <mergeCell ref="AV4:AW4"/>
-    <mergeCell ref="Z3:AA3"/>
-    <mergeCell ref="AX3:AY3"/>
-    <mergeCell ref="X3:Y3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7743,7 +7743,7 @@
       <c r="AH1" s="253"/>
     </row>
     <row r="2" spans="1:34" ht="19.95" customHeight="1">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="261" t="s">
         <v>1032</v>
       </c>
       <c r="B2" s="253"/>
@@ -8909,7 +8909,7 @@
       <c r="J1" s="253"/>
     </row>
     <row r="2" spans="1:10" ht="19.95" customHeight="1">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="261" t="s">
         <v>1079</v>
       </c>
       <c r="B2" s="253"/>
@@ -8923,49 +8923,49 @@
       <c r="J2" s="253"/>
     </row>
     <row r="4" spans="1:10" ht="24" customHeight="1">
-      <c r="A4" s="284" t="s">
+      <c r="A4" s="289" t="s">
         <v>1080</v>
       </c>
       <c r="B4" s="253"/>
-      <c r="C4" s="284" t="s">
+      <c r="C4" s="289" t="s">
         <v>1081</v>
       </c>
       <c r="D4" s="253"/>
-      <c r="E4" s="284" t="s">
+      <c r="E4" s="289" t="s">
         <v>1082</v>
       </c>
       <c r="F4" s="253"/>
-      <c r="G4" s="284" t="s">
+      <c r="G4" s="289" t="s">
         <v>1083</v>
       </c>
       <c r="H4" s="253"/>
-      <c r="I4" s="284" t="s">
+      <c r="I4" s="289" t="s">
         <v>1084</v>
       </c>
       <c r="J4" s="253"/>
     </row>
     <row r="5" spans="1:10" ht="42" customHeight="1">
-      <c r="A5" s="286" t="str">
+      <c r="A5" s="285" t="str">
         <f>IFERROR(INDEX(Ranking!$I$4:$I$7,MATCH(1,Ranking!$P$4:$P$7,0)),"?")</f>
         <v>Pedro Brandao</v>
       </c>
       <c r="B5" s="253"/>
-      <c r="C5" s="285">
+      <c r="C5" s="284">
         <f>IFERROR(MAX(Ranking!$M$4:$M$7),0)</f>
         <v>0</v>
       </c>
       <c r="D5" s="253"/>
-      <c r="E5" s="288">
+      <c r="E5" s="287">
         <f>COUNTIF('Jogos - Grupos'!H3:H74,"Finalizado")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F5" s="253"/>
-      <c r="G5" s="287">
+      <c r="G5" s="286">
         <f>COUNTIF('Mata-Mata - Jogos'!I4:I35,"Finalizado")</f>
         <v>0</v>
       </c>
       <c r="H5" s="253"/>
-      <c r="I5" s="289" t="s">
+      <c r="I5" s="288" t="s">
         <v>1077</v>
       </c>
       <c r="J5" s="253"/>
@@ -9116,11 +9116,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="I5:J5"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="A1:J1"/>
@@ -9128,6 +9123,11 @@
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="I5:J5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9522,11 +9522,15 @@
       <c r="E16" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="F16" s="10">
+        <v>0</v>
+      </c>
+      <c r="G16" s="10">
+        <v>1</v>
+      </c>
       <c r="H16" s="21" t="str">
         <f t="shared" si="0"/>
-        <v>Aguardando</v>
+        <v>Finalizado</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -9664,11 +9668,15 @@
       <c r="E22" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
+      <c r="F22" s="10">
+        <v>2</v>
+      </c>
+      <c r="G22" s="10">
+        <v>0</v>
+      </c>
       <c r="H22" s="26" t="str">
         <f t="shared" si="0"/>
-        <v>Aguardando</v>
+        <v>Finalizado</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -11037,7 +11045,7 @@
       <c r="EO1" s="253"/>
     </row>
     <row r="2" spans="1:145" ht="19.95" customHeight="1">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="261" t="s">
         <v>186</v>
       </c>
       <c r="B2" s="253"/>
@@ -11189,219 +11197,219 @@
       <c r="A3" s="67" t="s">
         <v>187</v>
       </c>
-      <c r="B3" s="256" t="s">
+      <c r="B3" s="263" t="s">
         <v>188</v>
       </c>
       <c r="C3" s="253"/>
-      <c r="D3" s="256" t="s">
+      <c r="D3" s="263" t="s">
         <v>189</v>
       </c>
       <c r="E3" s="253"/>
-      <c r="F3" s="256" t="s">
+      <c r="F3" s="263" t="s">
         <v>190</v>
       </c>
       <c r="G3" s="253"/>
-      <c r="H3" s="256" t="s">
+      <c r="H3" s="263" t="s">
         <v>191</v>
       </c>
       <c r="I3" s="253"/>
-      <c r="J3" s="256" t="s">
+      <c r="J3" s="263" t="s">
         <v>192</v>
       </c>
       <c r="K3" s="253"/>
-      <c r="L3" s="256" t="s">
+      <c r="L3" s="263" t="s">
         <v>193</v>
       </c>
       <c r="M3" s="253"/>
-      <c r="N3" s="260" t="s">
+      <c r="N3" s="264" t="s">
         <v>194</v>
       </c>
       <c r="O3" s="253"/>
-      <c r="P3" s="260" t="s">
+      <c r="P3" s="264" t="s">
         <v>195</v>
       </c>
       <c r="Q3" s="253"/>
-      <c r="R3" s="260" t="s">
+      <c r="R3" s="264" t="s">
         <v>196</v>
       </c>
       <c r="S3" s="253"/>
-      <c r="T3" s="260" t="s">
+      <c r="T3" s="264" t="s">
         <v>197</v>
       </c>
       <c r="U3" s="253"/>
-      <c r="V3" s="260" t="s">
+      <c r="V3" s="264" t="s">
         <v>198</v>
       </c>
       <c r="W3" s="253"/>
-      <c r="X3" s="260" t="s">
+      <c r="X3" s="264" t="s">
         <v>199</v>
       </c>
       <c r="Y3" s="253"/>
-      <c r="Z3" s="261" t="s">
+      <c r="Z3" s="259" t="s">
         <v>200</v>
       </c>
       <c r="AA3" s="253"/>
-      <c r="AB3" s="261" t="s">
+      <c r="AB3" s="259" t="s">
         <v>201</v>
       </c>
       <c r="AC3" s="253"/>
-      <c r="AD3" s="261" t="s">
+      <c r="AD3" s="259" t="s">
         <v>202</v>
       </c>
       <c r="AE3" s="253"/>
-      <c r="AF3" s="261" t="s">
+      <c r="AF3" s="259" t="s">
         <v>203</v>
       </c>
       <c r="AG3" s="253"/>
-      <c r="AH3" s="261" t="s">
+      <c r="AH3" s="259" t="s">
         <v>204</v>
       </c>
       <c r="AI3" s="253"/>
-      <c r="AJ3" s="261" t="s">
+      <c r="AJ3" s="259" t="s">
         <v>205</v>
       </c>
       <c r="AK3" s="253"/>
-      <c r="AL3" s="257" t="s">
+      <c r="AL3" s="260" t="s">
         <v>206</v>
       </c>
       <c r="AM3" s="253"/>
-      <c r="AN3" s="257" t="s">
+      <c r="AN3" s="260" t="s">
         <v>207</v>
       </c>
       <c r="AO3" s="253"/>
-      <c r="AP3" s="257" t="s">
+      <c r="AP3" s="260" t="s">
         <v>208</v>
       </c>
       <c r="AQ3" s="253"/>
-      <c r="AR3" s="257" t="s">
+      <c r="AR3" s="260" t="s">
         <v>209</v>
       </c>
       <c r="AS3" s="253"/>
-      <c r="AT3" s="257" t="s">
+      <c r="AT3" s="260" t="s">
         <v>210</v>
       </c>
       <c r="AU3" s="253"/>
-      <c r="AV3" s="257" t="s">
+      <c r="AV3" s="260" t="s">
         <v>211</v>
       </c>
       <c r="AW3" s="253"/>
-      <c r="AX3" s="258" t="s">
+      <c r="AX3" s="265" t="s">
         <v>212</v>
       </c>
       <c r="AY3" s="253"/>
-      <c r="AZ3" s="258" t="s">
+      <c r="AZ3" s="265" t="s">
         <v>213</v>
       </c>
       <c r="BA3" s="253"/>
-      <c r="BB3" s="258" t="s">
+      <c r="BB3" s="265" t="s">
         <v>214</v>
       </c>
       <c r="BC3" s="253"/>
-      <c r="BD3" s="258" t="s">
+      <c r="BD3" s="265" t="s">
         <v>215</v>
       </c>
       <c r="BE3" s="253"/>
-      <c r="BF3" s="258" t="s">
+      <c r="BF3" s="265" t="s">
         <v>216</v>
       </c>
       <c r="BG3" s="253"/>
-      <c r="BH3" s="258" t="s">
+      <c r="BH3" s="265" t="s">
         <v>217</v>
       </c>
       <c r="BI3" s="253"/>
-      <c r="BJ3" s="262" t="s">
+      <c r="BJ3" s="266" t="s">
         <v>218</v>
       </c>
       <c r="BK3" s="253"/>
-      <c r="BL3" s="262" t="s">
+      <c r="BL3" s="266" t="s">
         <v>219</v>
       </c>
       <c r="BM3" s="253"/>
-      <c r="BN3" s="262" t="s">
+      <c r="BN3" s="266" t="s">
         <v>220</v>
       </c>
       <c r="BO3" s="253"/>
-      <c r="BP3" s="262" t="s">
+      <c r="BP3" s="266" t="s">
         <v>221</v>
       </c>
       <c r="BQ3" s="253"/>
-      <c r="BR3" s="262" t="s">
+      <c r="BR3" s="266" t="s">
         <v>222</v>
       </c>
       <c r="BS3" s="253"/>
-      <c r="BT3" s="262" t="s">
+      <c r="BT3" s="266" t="s">
         <v>223</v>
       </c>
       <c r="BU3" s="253"/>
-      <c r="BV3" s="263" t="s">
+      <c r="BV3" s="256" t="s">
         <v>224</v>
       </c>
       <c r="BW3" s="253"/>
-      <c r="BX3" s="263" t="s">
+      <c r="BX3" s="256" t="s">
         <v>225</v>
       </c>
       <c r="BY3" s="253"/>
-      <c r="BZ3" s="263" t="s">
+      <c r="BZ3" s="256" t="s">
         <v>226</v>
       </c>
       <c r="CA3" s="253"/>
-      <c r="CB3" s="263" t="s">
+      <c r="CB3" s="256" t="s">
         <v>227</v>
       </c>
       <c r="CC3" s="253"/>
-      <c r="CD3" s="263" t="s">
+      <c r="CD3" s="256" t="s">
         <v>228</v>
       </c>
       <c r="CE3" s="253"/>
-      <c r="CF3" s="263" t="s">
+      <c r="CF3" s="256" t="s">
         <v>229</v>
       </c>
       <c r="CG3" s="253"/>
-      <c r="CH3" s="259" t="s">
+      <c r="CH3" s="257" t="s">
         <v>230</v>
       </c>
       <c r="CI3" s="253"/>
-      <c r="CJ3" s="259" t="s">
+      <c r="CJ3" s="257" t="s">
         <v>231</v>
       </c>
       <c r="CK3" s="253"/>
-      <c r="CL3" s="259" t="s">
+      <c r="CL3" s="257" t="s">
         <v>232</v>
       </c>
       <c r="CM3" s="253"/>
-      <c r="CN3" s="259" t="s">
+      <c r="CN3" s="257" t="s">
         <v>233</v>
       </c>
       <c r="CO3" s="253"/>
-      <c r="CP3" s="259" t="s">
+      <c r="CP3" s="257" t="s">
         <v>234</v>
       </c>
       <c r="CQ3" s="253"/>
-      <c r="CR3" s="259" t="s">
+      <c r="CR3" s="257" t="s">
         <v>235</v>
       </c>
       <c r="CS3" s="253"/>
-      <c r="CT3" s="265" t="s">
+      <c r="CT3" s="258" t="s">
         <v>236</v>
       </c>
       <c r="CU3" s="253"/>
-      <c r="CV3" s="265" t="s">
+      <c r="CV3" s="258" t="s">
         <v>237</v>
       </c>
       <c r="CW3" s="253"/>
-      <c r="CX3" s="265" t="s">
+      <c r="CX3" s="258" t="s">
         <v>238</v>
       </c>
       <c r="CY3" s="253"/>
-      <c r="CZ3" s="265" t="s">
+      <c r="CZ3" s="258" t="s">
         <v>239</v>
       </c>
       <c r="DA3" s="253"/>
-      <c r="DB3" s="265" t="s">
+      <c r="DB3" s="258" t="s">
         <v>240</v>
       </c>
       <c r="DC3" s="253"/>
-      <c r="DD3" s="265" t="s">
+      <c r="DD3" s="258" t="s">
         <v>241</v>
       </c>
       <c r="DE3" s="253"/>
@@ -11429,51 +11437,51 @@
         <v>247</v>
       </c>
       <c r="DQ3" s="253"/>
-      <c r="DR3" s="266" t="s">
+      <c r="DR3" s="268" t="s">
         <v>248</v>
       </c>
       <c r="DS3" s="253"/>
-      <c r="DT3" s="266" t="s">
+      <c r="DT3" s="268" t="s">
         <v>249</v>
       </c>
       <c r="DU3" s="253"/>
-      <c r="DV3" s="266" t="s">
+      <c r="DV3" s="268" t="s">
         <v>250</v>
       </c>
       <c r="DW3" s="253"/>
-      <c r="DX3" s="266" t="s">
+      <c r="DX3" s="268" t="s">
         <v>251</v>
       </c>
       <c r="DY3" s="253"/>
-      <c r="DZ3" s="266" t="s">
+      <c r="DZ3" s="268" t="s">
         <v>252</v>
       </c>
       <c r="EA3" s="253"/>
-      <c r="EB3" s="266" t="s">
+      <c r="EB3" s="268" t="s">
         <v>253</v>
       </c>
       <c r="EC3" s="253"/>
-      <c r="ED3" s="264" t="s">
+      <c r="ED3" s="262" t="s">
         <v>254</v>
       </c>
       <c r="EE3" s="253"/>
-      <c r="EF3" s="264" t="s">
+      <c r="EF3" s="262" t="s">
         <v>255</v>
       </c>
       <c r="EG3" s="253"/>
-      <c r="EH3" s="264" t="s">
+      <c r="EH3" s="262" t="s">
         <v>256</v>
       </c>
       <c r="EI3" s="253"/>
-      <c r="EJ3" s="264" t="s">
+      <c r="EJ3" s="262" t="s">
         <v>257</v>
       </c>
       <c r="EK3" s="253"/>
-      <c r="EL3" s="264" t="s">
+      <c r="EL3" s="262" t="s">
         <v>258</v>
       </c>
       <c r="EM3" s="253"/>
-      <c r="EN3" s="264" t="s">
+      <c r="EN3" s="262" t="s">
         <v>259</v>
       </c>
       <c r="EO3" s="253"/>
@@ -12513,16 +12521,54 @@
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="BX3:BY3"/>
-    <mergeCell ref="CN3:CO3"/>
-    <mergeCell ref="CZ3:DA3"/>
-    <mergeCell ref="AD3:AE3"/>
-    <mergeCell ref="AF3:AG3"/>
-    <mergeCell ref="AH3:AI3"/>
-    <mergeCell ref="AN3:AO3"/>
-    <mergeCell ref="CH3:CI3"/>
-    <mergeCell ref="CD3:CE3"/>
-    <mergeCell ref="CT3:CU3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="AP3:AQ3"/>
+    <mergeCell ref="BB3:BC3"/>
+    <mergeCell ref="CJ3:CK3"/>
+    <mergeCell ref="CL3:CM3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="X3:Y3"/>
+    <mergeCell ref="Z3:AA3"/>
+    <mergeCell ref="BT3:BU3"/>
+    <mergeCell ref="AJ3:AK3"/>
+    <mergeCell ref="AL3:AM3"/>
+    <mergeCell ref="CF3:CG3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="AR3:AS3"/>
+    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="EN3:EO3"/>
+    <mergeCell ref="CX3:CY3"/>
+    <mergeCell ref="DV3:DW3"/>
+    <mergeCell ref="EB3:EC3"/>
+    <mergeCell ref="ED3:EE3"/>
+    <mergeCell ref="EH3:EI3"/>
+    <mergeCell ref="DZ3:EA3"/>
+    <mergeCell ref="EF3:EG3"/>
+    <mergeCell ref="DH3:DI3"/>
+    <mergeCell ref="DT3:DU3"/>
+    <mergeCell ref="DR3:DS3"/>
+    <mergeCell ref="DX3:DY3"/>
+    <mergeCell ref="DD3:DE3"/>
+    <mergeCell ref="DF3:DG3"/>
+    <mergeCell ref="DB3:DC3"/>
+    <mergeCell ref="DN3:DO3"/>
+    <mergeCell ref="A1:EO1"/>
+    <mergeCell ref="AT3:AU3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="AV3:AW3"/>
+    <mergeCell ref="BD3:BE3"/>
+    <mergeCell ref="BF3:BG3"/>
+    <mergeCell ref="BH3:BI3"/>
+    <mergeCell ref="BN3:BO3"/>
+    <mergeCell ref="BP3:BQ3"/>
+    <mergeCell ref="BR3:BS3"/>
+    <mergeCell ref="DP3:DQ3"/>
+    <mergeCell ref="BZ3:CA3"/>
+    <mergeCell ref="CP3:CQ3"/>
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="AB3:AC3"/>
+    <mergeCell ref="CR3:CS3"/>
     <mergeCell ref="A2:EO2"/>
     <mergeCell ref="EJ3:EK3"/>
     <mergeCell ref="D3:E3"/>
@@ -12539,54 +12585,16 @@
     <mergeCell ref="DJ3:DK3"/>
     <mergeCell ref="EL3:EM3"/>
     <mergeCell ref="CV3:CW3"/>
-    <mergeCell ref="A1:EO1"/>
-    <mergeCell ref="AT3:AU3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="AV3:AW3"/>
-    <mergeCell ref="BD3:BE3"/>
-    <mergeCell ref="BF3:BG3"/>
-    <mergeCell ref="BH3:BI3"/>
-    <mergeCell ref="BN3:BO3"/>
-    <mergeCell ref="BP3:BQ3"/>
-    <mergeCell ref="BR3:BS3"/>
-    <mergeCell ref="DP3:DQ3"/>
-    <mergeCell ref="BZ3:CA3"/>
-    <mergeCell ref="CP3:CQ3"/>
-    <mergeCell ref="V3:W3"/>
-    <mergeCell ref="AB3:AC3"/>
-    <mergeCell ref="CR3:CS3"/>
-    <mergeCell ref="EN3:EO3"/>
-    <mergeCell ref="CX3:CY3"/>
-    <mergeCell ref="DV3:DW3"/>
-    <mergeCell ref="EB3:EC3"/>
-    <mergeCell ref="ED3:EE3"/>
-    <mergeCell ref="EH3:EI3"/>
-    <mergeCell ref="DZ3:EA3"/>
-    <mergeCell ref="EF3:EG3"/>
-    <mergeCell ref="DH3:DI3"/>
-    <mergeCell ref="DT3:DU3"/>
-    <mergeCell ref="DR3:DS3"/>
-    <mergeCell ref="DX3:DY3"/>
-    <mergeCell ref="DD3:DE3"/>
-    <mergeCell ref="DF3:DG3"/>
-    <mergeCell ref="DB3:DC3"/>
-    <mergeCell ref="DN3:DO3"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="AP3:AQ3"/>
-    <mergeCell ref="BB3:BC3"/>
-    <mergeCell ref="CJ3:CK3"/>
-    <mergeCell ref="CL3:CM3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="X3:Y3"/>
-    <mergeCell ref="Z3:AA3"/>
-    <mergeCell ref="BT3:BU3"/>
-    <mergeCell ref="AJ3:AK3"/>
-    <mergeCell ref="AL3:AM3"/>
-    <mergeCell ref="CF3:CG3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="AR3:AS3"/>
-    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="BX3:BY3"/>
+    <mergeCell ref="CN3:CO3"/>
+    <mergeCell ref="CZ3:DA3"/>
+    <mergeCell ref="AD3:AE3"/>
+    <mergeCell ref="AF3:AG3"/>
+    <mergeCell ref="AH3:AI3"/>
+    <mergeCell ref="AN3:AO3"/>
+    <mergeCell ref="CH3:CI3"/>
+    <mergeCell ref="CD3:CE3"/>
+    <mergeCell ref="CT3:CU3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12612,7 +12620,7 @@
       <c r="C1" s="253"/>
     </row>
     <row r="2" spans="1:3" ht="19.95" customHeight="1">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="261" t="s">
         <v>266</v>
       </c>
       <c r="B2" s="253"/>
@@ -12765,7 +12773,7 @@
       <c r="BV1" s="253"/>
     </row>
     <row r="2" spans="1:74" ht="19.95" customHeight="1">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="261" t="s">
         <v>271</v>
       </c>
       <c r="B2" s="253"/>
@@ -13344,9 +13352,9 @@
         <f>IF(OR('Jogos - Grupos'!F15="",'Jogos - Grupos'!G15=""),"-",IF(OR('Apostas - Grupos'!Z5="",'Apostas - Grupos'!AA5=""),0,IF(AND('Apostas - Grupos'!Z5='Jogos - Grupos'!F15,'Apostas - Grupos'!AA5='Jogos - Grupos'!G15),5,IF(OR(AND('Jogos - Grupos'!F15='Jogos - Grupos'!G15,'Apostas - Grupos'!Z5='Apostas - Grupos'!AA5),AND('Jogos - Grupos'!F15&gt;'Jogos - Grupos'!G15,'Apostas - Grupos'!Z5&gt;'Apostas - Grupos'!AA5),AND('Jogos - Grupos'!F15&lt;'Jogos - Grupos'!G15,'Apostas - Grupos'!Z5&lt;'Apostas - Grupos'!AA5)),IF(('Apostas - Grupos'!Z5-'Apostas - Grupos'!AA5)=('Jogos - Grupos'!F15-'Jogos - Grupos'!G15),3,2),0))))</f>
         <v>0</v>
       </c>
-      <c r="O5" s="106" t="str">
+      <c r="O5" s="106">
         <f>IF(OR('Jogos - Grupos'!F16="",'Jogos - Grupos'!G16=""),"-",IF(OR('Apostas - Grupos'!AB5="",'Apostas - Grupos'!AC5=""),0,IF(AND('Apostas - Grupos'!AB5='Jogos - Grupos'!F16,'Apostas - Grupos'!AC5='Jogos - Grupos'!G16),5,IF(OR(AND('Jogos - Grupos'!F16='Jogos - Grupos'!G16,'Apostas - Grupos'!AB5='Apostas - Grupos'!AC5),AND('Jogos - Grupos'!F16&gt;'Jogos - Grupos'!G16,'Apostas - Grupos'!AB5&gt;'Apostas - Grupos'!AC5),AND('Jogos - Grupos'!F16&lt;'Jogos - Grupos'!G16,'Apostas - Grupos'!AB5&lt;'Apostas - Grupos'!AC5)),IF(('Apostas - Grupos'!AB5-'Apostas - Grupos'!AC5)=('Jogos - Grupos'!F16-'Jogos - Grupos'!G16),3,2),0))))</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="P5" s="106" t="str">
         <f>IF(OR('Jogos - Grupos'!F17="",'Jogos - Grupos'!G17=""),"-",IF(OR('Apostas - Grupos'!AD5="",'Apostas - Grupos'!AE5=""),0,IF(AND('Apostas - Grupos'!AD5='Jogos - Grupos'!F17,'Apostas - Grupos'!AE5='Jogos - Grupos'!G17),5,IF(OR(AND('Jogos - Grupos'!F17='Jogos - Grupos'!G17,'Apostas - Grupos'!AD5='Apostas - Grupos'!AE5),AND('Jogos - Grupos'!F17&gt;'Jogos - Grupos'!G17,'Apostas - Grupos'!AD5&gt;'Apostas - Grupos'!AE5),AND('Jogos - Grupos'!F17&lt;'Jogos - Grupos'!G17,'Apostas - Grupos'!AD5&lt;'Apostas - Grupos'!AE5)),IF(('Apostas - Grupos'!AD5-'Apostas - Grupos'!AE5)=('Jogos - Grupos'!F17-'Jogos - Grupos'!G17),3,2),0))))</f>
@@ -13368,9 +13376,9 @@
         <f>IF(OR('Jogos - Grupos'!F21="",'Jogos - Grupos'!G21=""),"-",IF(OR('Apostas - Grupos'!AL5="",'Apostas - Grupos'!AM5=""),0,IF(AND('Apostas - Grupos'!AL5='Jogos - Grupos'!F21,'Apostas - Grupos'!AM5='Jogos - Grupos'!G21),5,IF(OR(AND('Jogos - Grupos'!F21='Jogos - Grupos'!G21,'Apostas - Grupos'!AL5='Apostas - Grupos'!AM5),AND('Jogos - Grupos'!F21&gt;'Jogos - Grupos'!G21,'Apostas - Grupos'!AL5&gt;'Apostas - Grupos'!AM5),AND('Jogos - Grupos'!F21&lt;'Jogos - Grupos'!G21,'Apostas - Grupos'!AL5&lt;'Apostas - Grupos'!AM5)),IF(('Apostas - Grupos'!AL5-'Apostas - Grupos'!AM5)=('Jogos - Grupos'!F21-'Jogos - Grupos'!G21),3,2),0))))</f>
         <v>0</v>
       </c>
-      <c r="U5" s="106" t="str">
+      <c r="U5" s="106">
         <f>IF(OR('Jogos - Grupos'!F22="",'Jogos - Grupos'!G22=""),"-",IF(OR('Apostas - Grupos'!AN5="",'Apostas - Grupos'!AO5=""),0,IF(AND('Apostas - Grupos'!AN5='Jogos - Grupos'!F22,'Apostas - Grupos'!AO5='Jogos - Grupos'!G22),5,IF(OR(AND('Jogos - Grupos'!F22='Jogos - Grupos'!G22,'Apostas - Grupos'!AN5='Apostas - Grupos'!AO5),AND('Jogos - Grupos'!F22&gt;'Jogos - Grupos'!G22,'Apostas - Grupos'!AN5&gt;'Apostas - Grupos'!AO5),AND('Jogos - Grupos'!F22&lt;'Jogos - Grupos'!G22,'Apostas - Grupos'!AN5&lt;'Apostas - Grupos'!AO5)),IF(('Apostas - Grupos'!AN5-'Apostas - Grupos'!AO5)=('Jogos - Grupos'!F22-'Jogos - Grupos'!G22),3,2),0))))</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="V5" s="106" t="str">
         <f>IF(OR('Jogos - Grupos'!F23="",'Jogos - Grupos'!G23=""),"-",IF(OR('Apostas - Grupos'!AP5="",'Apostas - Grupos'!AQ5=""),0,IF(AND('Apostas - Grupos'!AP5='Jogos - Grupos'!F23,'Apostas - Grupos'!AQ5='Jogos - Grupos'!G23),5,IF(OR(AND('Jogos - Grupos'!F23='Jogos - Grupos'!G23,'Apostas - Grupos'!AP5='Apostas - Grupos'!AQ5),AND('Jogos - Grupos'!F23&gt;'Jogos - Grupos'!G23,'Apostas - Grupos'!AP5&gt;'Apostas - Grupos'!AQ5),AND('Jogos - Grupos'!F23&lt;'Jogos - Grupos'!G23,'Apostas - Grupos'!AP5&lt;'Apostas - Grupos'!AQ5)),IF(('Apostas - Grupos'!AP5-'Apostas - Grupos'!AQ5)=('Jogos - Grupos'!F23-'Jogos - Grupos'!G23),3,2),0))))</f>
@@ -13641,9 +13649,9 @@
         <f>IF(OR('Jogos - Grupos'!F15="",'Jogos - Grupos'!G15=""),"-",IF(OR('Apostas - Grupos'!Z6="",'Apostas - Grupos'!AA6=""),0,IF(AND('Apostas - Grupos'!Z6='Jogos - Grupos'!F15,'Apostas - Grupos'!AA6='Jogos - Grupos'!G15),5,IF(OR(AND('Jogos - Grupos'!F15='Jogos - Grupos'!G15,'Apostas - Grupos'!Z6='Apostas - Grupos'!AA6),AND('Jogos - Grupos'!F15&gt;'Jogos - Grupos'!G15,'Apostas - Grupos'!Z6&gt;'Apostas - Grupos'!AA6),AND('Jogos - Grupos'!F15&lt;'Jogos - Grupos'!G15,'Apostas - Grupos'!Z6&lt;'Apostas - Grupos'!AA6)),IF(('Apostas - Grupos'!Z6-'Apostas - Grupos'!AA6)=('Jogos - Grupos'!F15-'Jogos - Grupos'!G15),3,2),0))))</f>
         <v>0</v>
       </c>
-      <c r="O6" s="108" t="str">
+      <c r="O6" s="108">
         <f>IF(OR('Jogos - Grupos'!F16="",'Jogos - Grupos'!G16=""),"-",IF(OR('Apostas - Grupos'!AB6="",'Apostas - Grupos'!AC6=""),0,IF(AND('Apostas - Grupos'!AB6='Jogos - Grupos'!F16,'Apostas - Grupos'!AC6='Jogos - Grupos'!G16),5,IF(OR(AND('Jogos - Grupos'!F16='Jogos - Grupos'!G16,'Apostas - Grupos'!AB6='Apostas - Grupos'!AC6),AND('Jogos - Grupos'!F16&gt;'Jogos - Grupos'!G16,'Apostas - Grupos'!AB6&gt;'Apostas - Grupos'!AC6),AND('Jogos - Grupos'!F16&lt;'Jogos - Grupos'!G16,'Apostas - Grupos'!AB6&lt;'Apostas - Grupos'!AC6)),IF(('Apostas - Grupos'!AB6-'Apostas - Grupos'!AC6)=('Jogos - Grupos'!F16-'Jogos - Grupos'!G16),3,2),0))))</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="P6" s="108" t="str">
         <f>IF(OR('Jogos - Grupos'!F17="",'Jogos - Grupos'!G17=""),"-",IF(OR('Apostas - Grupos'!AD6="",'Apostas - Grupos'!AE6=""),0,IF(AND('Apostas - Grupos'!AD6='Jogos - Grupos'!F17,'Apostas - Grupos'!AE6='Jogos - Grupos'!G17),5,IF(OR(AND('Jogos - Grupos'!F17='Jogos - Grupos'!G17,'Apostas - Grupos'!AD6='Apostas - Grupos'!AE6),AND('Jogos - Grupos'!F17&gt;'Jogos - Grupos'!G17,'Apostas - Grupos'!AD6&gt;'Apostas - Grupos'!AE6),AND('Jogos - Grupos'!F17&lt;'Jogos - Grupos'!G17,'Apostas - Grupos'!AD6&lt;'Apostas - Grupos'!AE6)),IF(('Apostas - Grupos'!AD6-'Apostas - Grupos'!AE6)=('Jogos - Grupos'!F17-'Jogos - Grupos'!G17),3,2),0))))</f>
@@ -13665,9 +13673,9 @@
         <f>IF(OR('Jogos - Grupos'!F21="",'Jogos - Grupos'!G21=""),"-",IF(OR('Apostas - Grupos'!AL6="",'Apostas - Grupos'!AM6=""),0,IF(AND('Apostas - Grupos'!AL6='Jogos - Grupos'!F21,'Apostas - Grupos'!AM6='Jogos - Grupos'!G21),5,IF(OR(AND('Jogos - Grupos'!F21='Jogos - Grupos'!G21,'Apostas - Grupos'!AL6='Apostas - Grupos'!AM6),AND('Jogos - Grupos'!F21&gt;'Jogos - Grupos'!G21,'Apostas - Grupos'!AL6&gt;'Apostas - Grupos'!AM6),AND('Jogos - Grupos'!F21&lt;'Jogos - Grupos'!G21,'Apostas - Grupos'!AL6&lt;'Apostas - Grupos'!AM6)),IF(('Apostas - Grupos'!AL6-'Apostas - Grupos'!AM6)=('Jogos - Grupos'!F21-'Jogos - Grupos'!G21),3,2),0))))</f>
         <v>0</v>
       </c>
-      <c r="U6" s="108" t="str">
+      <c r="U6" s="108">
         <f>IF(OR('Jogos - Grupos'!F22="",'Jogos - Grupos'!G22=""),"-",IF(OR('Apostas - Grupos'!AN6="",'Apostas - Grupos'!AO6=""),0,IF(AND('Apostas - Grupos'!AN6='Jogos - Grupos'!F22,'Apostas - Grupos'!AO6='Jogos - Grupos'!G22),5,IF(OR(AND('Jogos - Grupos'!F22='Jogos - Grupos'!G22,'Apostas - Grupos'!AN6='Apostas - Grupos'!AO6),AND('Jogos - Grupos'!F22&gt;'Jogos - Grupos'!G22,'Apostas - Grupos'!AN6&gt;'Apostas - Grupos'!AO6),AND('Jogos - Grupos'!F22&lt;'Jogos - Grupos'!G22,'Apostas - Grupos'!AN6&lt;'Apostas - Grupos'!AO6)),IF(('Apostas - Grupos'!AN6-'Apostas - Grupos'!AO6)=('Jogos - Grupos'!F22-'Jogos - Grupos'!G22),3,2),0))))</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="V6" s="108" t="str">
         <f>IF(OR('Jogos - Grupos'!F23="",'Jogos - Grupos'!G23=""),"-",IF(OR('Apostas - Grupos'!AP6="",'Apostas - Grupos'!AQ6=""),0,IF(AND('Apostas - Grupos'!AP6='Jogos - Grupos'!F23,'Apostas - Grupos'!AQ6='Jogos - Grupos'!G23),5,IF(OR(AND('Jogos - Grupos'!F23='Jogos - Grupos'!G23,'Apostas - Grupos'!AP6='Apostas - Grupos'!AQ6),AND('Jogos - Grupos'!F23&gt;'Jogos - Grupos'!G23,'Apostas - Grupos'!AP6&gt;'Apostas - Grupos'!AQ6),AND('Jogos - Grupos'!F23&lt;'Jogos - Grupos'!G23,'Apostas - Grupos'!AP6&lt;'Apostas - Grupos'!AQ6)),IF(('Apostas - Grupos'!AP6-'Apostas - Grupos'!AQ6)=('Jogos - Grupos'!F23-'Jogos - Grupos'!G23),3,2),0))))</f>
@@ -13938,9 +13946,9 @@
         <f>IF(OR('Jogos - Grupos'!F15="",'Jogos - Grupos'!G15=""),"-",IF(OR('Apostas - Grupos'!Z7="",'Apostas - Grupos'!AA7=""),0,IF(AND('Apostas - Grupos'!Z7='Jogos - Grupos'!F15,'Apostas - Grupos'!AA7='Jogos - Grupos'!G15),5,IF(OR(AND('Jogos - Grupos'!F15='Jogos - Grupos'!G15,'Apostas - Grupos'!Z7='Apostas - Grupos'!AA7),AND('Jogos - Grupos'!F15&gt;'Jogos - Grupos'!G15,'Apostas - Grupos'!Z7&gt;'Apostas - Grupos'!AA7),AND('Jogos - Grupos'!F15&lt;'Jogos - Grupos'!G15,'Apostas - Grupos'!Z7&lt;'Apostas - Grupos'!AA7)),IF(('Apostas - Grupos'!Z7-'Apostas - Grupos'!AA7)=('Jogos - Grupos'!F15-'Jogos - Grupos'!G15),3,2),0))))</f>
         <v>0</v>
       </c>
-      <c r="O7" s="106" t="str">
+      <c r="O7" s="106">
         <f>IF(OR('Jogos - Grupos'!F16="",'Jogos - Grupos'!G16=""),"-",IF(OR('Apostas - Grupos'!AB7="",'Apostas - Grupos'!AC7=""),0,IF(AND('Apostas - Grupos'!AB7='Jogos - Grupos'!F16,'Apostas - Grupos'!AC7='Jogos - Grupos'!G16),5,IF(OR(AND('Jogos - Grupos'!F16='Jogos - Grupos'!G16,'Apostas - Grupos'!AB7='Apostas - Grupos'!AC7),AND('Jogos - Grupos'!F16&gt;'Jogos - Grupos'!G16,'Apostas - Grupos'!AB7&gt;'Apostas - Grupos'!AC7),AND('Jogos - Grupos'!F16&lt;'Jogos - Grupos'!G16,'Apostas - Grupos'!AB7&lt;'Apostas - Grupos'!AC7)),IF(('Apostas - Grupos'!AB7-'Apostas - Grupos'!AC7)=('Jogos - Grupos'!F16-'Jogos - Grupos'!G16),3,2),0))))</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="P7" s="106" t="str">
         <f>IF(OR('Jogos - Grupos'!F17="",'Jogos - Grupos'!G17=""),"-",IF(OR('Apostas - Grupos'!AD7="",'Apostas - Grupos'!AE7=""),0,IF(AND('Apostas - Grupos'!AD7='Jogos - Grupos'!F17,'Apostas - Grupos'!AE7='Jogos - Grupos'!G17),5,IF(OR(AND('Jogos - Grupos'!F17='Jogos - Grupos'!G17,'Apostas - Grupos'!AD7='Apostas - Grupos'!AE7),AND('Jogos - Grupos'!F17&gt;'Jogos - Grupos'!G17,'Apostas - Grupos'!AD7&gt;'Apostas - Grupos'!AE7),AND('Jogos - Grupos'!F17&lt;'Jogos - Grupos'!G17,'Apostas - Grupos'!AD7&lt;'Apostas - Grupos'!AE7)),IF(('Apostas - Grupos'!AD7-'Apostas - Grupos'!AE7)=('Jogos - Grupos'!F17-'Jogos - Grupos'!G17),3,2),0))))</f>
@@ -13962,9 +13970,9 @@
         <f>IF(OR('Jogos - Grupos'!F21="",'Jogos - Grupos'!G21=""),"-",IF(OR('Apostas - Grupos'!AL7="",'Apostas - Grupos'!AM7=""),0,IF(AND('Apostas - Grupos'!AL7='Jogos - Grupos'!F21,'Apostas - Grupos'!AM7='Jogos - Grupos'!G21),5,IF(OR(AND('Jogos - Grupos'!F21='Jogos - Grupos'!G21,'Apostas - Grupos'!AL7='Apostas - Grupos'!AM7),AND('Jogos - Grupos'!F21&gt;'Jogos - Grupos'!G21,'Apostas - Grupos'!AL7&gt;'Apostas - Grupos'!AM7),AND('Jogos - Grupos'!F21&lt;'Jogos - Grupos'!G21,'Apostas - Grupos'!AL7&lt;'Apostas - Grupos'!AM7)),IF(('Apostas - Grupos'!AL7-'Apostas - Grupos'!AM7)=('Jogos - Grupos'!F21-'Jogos - Grupos'!G21),3,2),0))))</f>
         <v>0</v>
       </c>
-      <c r="U7" s="106" t="str">
+      <c r="U7" s="106">
         <f>IF(OR('Jogos - Grupos'!F22="",'Jogos - Grupos'!G22=""),"-",IF(OR('Apostas - Grupos'!AN7="",'Apostas - Grupos'!AO7=""),0,IF(AND('Apostas - Grupos'!AN7='Jogos - Grupos'!F22,'Apostas - Grupos'!AO7='Jogos - Grupos'!G22),5,IF(OR(AND('Jogos - Grupos'!F22='Jogos - Grupos'!G22,'Apostas - Grupos'!AN7='Apostas - Grupos'!AO7),AND('Jogos - Grupos'!F22&gt;'Jogos - Grupos'!G22,'Apostas - Grupos'!AN7&gt;'Apostas - Grupos'!AO7),AND('Jogos - Grupos'!F22&lt;'Jogos - Grupos'!G22,'Apostas - Grupos'!AN7&lt;'Apostas - Grupos'!AO7)),IF(('Apostas - Grupos'!AN7-'Apostas - Grupos'!AO7)=('Jogos - Grupos'!F22-'Jogos - Grupos'!G22),3,2),0))))</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="V7" s="106" t="str">
         <f>IF(OR('Jogos - Grupos'!F23="",'Jogos - Grupos'!G23=""),"-",IF(OR('Apostas - Grupos'!AP7="",'Apostas - Grupos'!AQ7=""),0,IF(AND('Apostas - Grupos'!AP7='Jogos - Grupos'!F23,'Apostas - Grupos'!AQ7='Jogos - Grupos'!G23),5,IF(OR(AND('Jogos - Grupos'!F23='Jogos - Grupos'!G23,'Apostas - Grupos'!AP7='Apostas - Grupos'!AQ7),AND('Jogos - Grupos'!F23&gt;'Jogos - Grupos'!G23,'Apostas - Grupos'!AP7&gt;'Apostas - Grupos'!AQ7),AND('Jogos - Grupos'!F23&lt;'Jogos - Grupos'!G23,'Apostas - Grupos'!AP7&lt;'Apostas - Grupos'!AQ7)),IF(('Apostas - Grupos'!AP7-'Apostas - Grupos'!AQ7)=('Jogos - Grupos'!F23-'Jogos - Grupos'!G23),3,2),0))))</f>
@@ -14235,9 +14243,9 @@
         <f>IF(OR('Jogos - Grupos'!F15="",'Jogos - Grupos'!G15=""),"-",IF(OR('Apostas - Grupos'!Z8="",'Apostas - Grupos'!AA8=""),0,IF(AND('Apostas - Grupos'!Z8='Jogos - Grupos'!F15,'Apostas - Grupos'!AA8='Jogos - Grupos'!G15),5,IF(OR(AND('Jogos - Grupos'!F15='Jogos - Grupos'!G15,'Apostas - Grupos'!Z8='Apostas - Grupos'!AA8),AND('Jogos - Grupos'!F15&gt;'Jogos - Grupos'!G15,'Apostas - Grupos'!Z8&gt;'Apostas - Grupos'!AA8),AND('Jogos - Grupos'!F15&lt;'Jogos - Grupos'!G15,'Apostas - Grupos'!Z8&lt;'Apostas - Grupos'!AA8)),IF(('Apostas - Grupos'!Z8-'Apostas - Grupos'!AA8)=('Jogos - Grupos'!F15-'Jogos - Grupos'!G15),3,2),0))))</f>
         <v>0</v>
       </c>
-      <c r="O8" s="108" t="str">
+      <c r="O8" s="108">
         <f>IF(OR('Jogos - Grupos'!F16="",'Jogos - Grupos'!G16=""),"-",IF(OR('Apostas - Grupos'!AB8="",'Apostas - Grupos'!AC8=""),0,IF(AND('Apostas - Grupos'!AB8='Jogos - Grupos'!F16,'Apostas - Grupos'!AC8='Jogos - Grupos'!G16),5,IF(OR(AND('Jogos - Grupos'!F16='Jogos - Grupos'!G16,'Apostas - Grupos'!AB8='Apostas - Grupos'!AC8),AND('Jogos - Grupos'!F16&gt;'Jogos - Grupos'!G16,'Apostas - Grupos'!AB8&gt;'Apostas - Grupos'!AC8),AND('Jogos - Grupos'!F16&lt;'Jogos - Grupos'!G16,'Apostas - Grupos'!AB8&lt;'Apostas - Grupos'!AC8)),IF(('Apostas - Grupos'!AB8-'Apostas - Grupos'!AC8)=('Jogos - Grupos'!F16-'Jogos - Grupos'!G16),3,2),0))))</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="P8" s="108" t="str">
         <f>IF(OR('Jogos - Grupos'!F17="",'Jogos - Grupos'!G17=""),"-",IF(OR('Apostas - Grupos'!AD8="",'Apostas - Grupos'!AE8=""),0,IF(AND('Apostas - Grupos'!AD8='Jogos - Grupos'!F17,'Apostas - Grupos'!AE8='Jogos - Grupos'!G17),5,IF(OR(AND('Jogos - Grupos'!F17='Jogos - Grupos'!G17,'Apostas - Grupos'!AD8='Apostas - Grupos'!AE8),AND('Jogos - Grupos'!F17&gt;'Jogos - Grupos'!G17,'Apostas - Grupos'!AD8&gt;'Apostas - Grupos'!AE8),AND('Jogos - Grupos'!F17&lt;'Jogos - Grupos'!G17,'Apostas - Grupos'!AD8&lt;'Apostas - Grupos'!AE8)),IF(('Apostas - Grupos'!AD8-'Apostas - Grupos'!AE8)=('Jogos - Grupos'!F17-'Jogos - Grupos'!G17),3,2),0))))</f>
@@ -14259,9 +14267,9 @@
         <f>IF(OR('Jogos - Grupos'!F21="",'Jogos - Grupos'!G21=""),"-",IF(OR('Apostas - Grupos'!AL8="",'Apostas - Grupos'!AM8=""),0,IF(AND('Apostas - Grupos'!AL8='Jogos - Grupos'!F21,'Apostas - Grupos'!AM8='Jogos - Grupos'!G21),5,IF(OR(AND('Jogos - Grupos'!F21='Jogos - Grupos'!G21,'Apostas - Grupos'!AL8='Apostas - Grupos'!AM8),AND('Jogos - Grupos'!F21&gt;'Jogos - Grupos'!G21,'Apostas - Grupos'!AL8&gt;'Apostas - Grupos'!AM8),AND('Jogos - Grupos'!F21&lt;'Jogos - Grupos'!G21,'Apostas - Grupos'!AL8&lt;'Apostas - Grupos'!AM8)),IF(('Apostas - Grupos'!AL8-'Apostas - Grupos'!AM8)=('Jogos - Grupos'!F21-'Jogos - Grupos'!G21),3,2),0))))</f>
         <v>0</v>
       </c>
-      <c r="U8" s="108" t="str">
+      <c r="U8" s="108">
         <f>IF(OR('Jogos - Grupos'!F22="",'Jogos - Grupos'!G22=""),"-",IF(OR('Apostas - Grupos'!AN8="",'Apostas - Grupos'!AO8=""),0,IF(AND('Apostas - Grupos'!AN8='Jogos - Grupos'!F22,'Apostas - Grupos'!AO8='Jogos - Grupos'!G22),5,IF(OR(AND('Jogos - Grupos'!F22='Jogos - Grupos'!G22,'Apostas - Grupos'!AN8='Apostas - Grupos'!AO8),AND('Jogos - Grupos'!F22&gt;'Jogos - Grupos'!G22,'Apostas - Grupos'!AN8&gt;'Apostas - Grupos'!AO8),AND('Jogos - Grupos'!F22&lt;'Jogos - Grupos'!G22,'Apostas - Grupos'!AN8&lt;'Apostas - Grupos'!AO8)),IF(('Apostas - Grupos'!AN8-'Apostas - Grupos'!AO8)=('Jogos - Grupos'!F22-'Jogos - Grupos'!G22),3,2),0))))</f>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="V8" s="108" t="str">
         <f>IF(OR('Jogos - Grupos'!F23="",'Jogos - Grupos'!G23=""),"-",IF(OR('Apostas - Grupos'!AP8="",'Apostas - Grupos'!AQ8=""),0,IF(AND('Apostas - Grupos'!AP8='Jogos - Grupos'!F23,'Apostas - Grupos'!AQ8='Jogos - Grupos'!G23),5,IF(OR(AND('Jogos - Grupos'!F23='Jogos - Grupos'!G23,'Apostas - Grupos'!AP8='Apostas - Grupos'!AQ8),AND('Jogos - Grupos'!F23&gt;'Jogos - Grupos'!G23,'Apostas - Grupos'!AP8&gt;'Apostas - Grupos'!AQ8),AND('Jogos - Grupos'!F23&lt;'Jogos - Grupos'!G23,'Apostas - Grupos'!AP8&lt;'Apostas - Grupos'!AQ8)),IF(('Apostas - Grupos'!AP8-'Apostas - Grupos'!AQ8)=('Jogos - Grupos'!F23-'Jogos - Grupos'!G23),3,2),0))))</f>
@@ -14949,7 +14957,7 @@
       </c>
       <c r="J11" s="19">
         <f>RANK(I11,$I$11:$I$14,0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" s="114">
         <v>5</v>
@@ -14992,7 +15000,7 @@
       </c>
       <c r="J12" s="19">
         <f>RANK(I12,$I$11:$I$14,0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" s="114">
         <v>14</v>
@@ -15019,11 +15027,11 @@
       </c>
       <c r="F13" s="114">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A13)*('Jogos - Grupos'!$D$3:$D$74=$B13)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*'Jogos - Grupos'!$G$3:$G$74)+SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A13)*('Jogos - Grupos'!$E$3:$E$74=$B13)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*'Jogos - Grupos'!$F$3:$F$74)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="114">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H13" s="19">
         <f t="shared" si="1"/>
@@ -15031,7 +15039,7 @@
       </c>
       <c r="I13" s="114">
         <f t="shared" si="2"/>
-        <v>200000414</v>
+        <v>199000414</v>
       </c>
       <c r="J13" s="19">
         <f>RANK(I13,$I$11:$I$14,0)</f>
@@ -15050,7 +15058,7 @@
       </c>
       <c r="C14" s="114">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A14)*('Jogos - Grupos'!$D$3:$D$74=$B14)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*('Jogos - Grupos'!$F$3:$F$74&gt;'Jogos - Grupos'!$G$3:$G$74))+SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A14)*('Jogos - Grupos'!$E$3:$E$74=$B14)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*('Jogos - Grupos'!$G$3:$G$74&gt;'Jogos - Grupos'!$F$3:$F$74))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="114">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A14)*(('Jogos - Grupos'!$D$3:$D$74=$B14)+('Jogos - Grupos'!$E$3:$E$74=$B14))*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*('Jogos - Grupos'!$F$3:$F$74='Jogos - Grupos'!$G$3:$G$74))</f>
@@ -15058,7 +15066,7 @@
       </c>
       <c r="E14" s="114">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A14)*('Jogos - Grupos'!$D$3:$D$74=$B14)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*'Jogos - Grupos'!$F$3:$F$74)+SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A14)*('Jogos - Grupos'!$E$3:$E$74=$B14)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*'Jogos - Grupos'!$G$3:$G$74)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="114">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A14)*('Jogos - Grupos'!$D$3:$D$74=$B14)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*'Jogos - Grupos'!$G$3:$G$74)+SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A14)*('Jogos - Grupos'!$E$3:$E$74=$B14)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*'Jogos - Grupos'!$F$3:$F$74)</f>
@@ -15066,19 +15074,19 @@
       </c>
       <c r="G14" s="114">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="19">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I14" s="114">
         <f t="shared" si="2"/>
-        <v>200000473</v>
+        <v>3201001473</v>
       </c>
       <c r="J14" s="19">
         <f>RANK(I14,$I$11:$I$14,0)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K14" s="114">
         <v>27</v>
@@ -15179,7 +15187,7 @@
       </c>
       <c r="C17" s="116">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A17)*('Jogos - Grupos'!$D$3:$D$74=$B17)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*('Jogos - Grupos'!$F$3:$F$74&gt;'Jogos - Grupos'!$G$3:$G$74))+SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A17)*('Jogos - Grupos'!$E$3:$E$74=$B17)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*('Jogos - Grupos'!$G$3:$G$74&gt;'Jogos - Grupos'!$F$3:$F$74))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="116">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A17)*(('Jogos - Grupos'!$D$3:$D$74=$B17)+('Jogos - Grupos'!$E$3:$E$74=$B17))*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*('Jogos - Grupos'!$F$3:$F$74='Jogos - Grupos'!$G$3:$G$74))</f>
@@ -15187,7 +15195,7 @@
       </c>
       <c r="E17" s="116">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A17)*('Jogos - Grupos'!$D$3:$D$74=$B17)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*'Jogos - Grupos'!$F$3:$F$74)+SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A17)*('Jogos - Grupos'!$E$3:$E$74=$B17)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*'Jogos - Grupos'!$G$3:$G$74)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F17" s="116">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A17)*('Jogos - Grupos'!$D$3:$D$74=$B17)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*'Jogos - Grupos'!$G$3:$G$74)+SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A17)*('Jogos - Grupos'!$E$3:$E$74=$B17)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*'Jogos - Grupos'!$F$3:$F$74)</f>
@@ -15195,15 +15203,15 @@
       </c>
       <c r="G17" s="116">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H17" s="24">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I17" s="116">
         <f t="shared" si="2"/>
-        <v>200000477</v>
+        <v>3202002477</v>
       </c>
       <c r="J17" s="24">
         <f>RANK(I17,$I$15:$I$18,0)</f>
@@ -15234,11 +15242,11 @@
       </c>
       <c r="F18" s="116">
         <f>SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A18)*('Jogos - Grupos'!$D$3:$D$74=$B18)*ISNUMBER('Jogos - Grupos'!$G$3:$G$74)*'Jogos - Grupos'!$G$3:$G$74)+SUMPRODUCT(('Jogos - Grupos'!$C$3:$C$74=$A18)*('Jogos - Grupos'!$E$3:$E$74=$B18)*ISNUMBER('Jogos - Grupos'!$F$3:$F$74)*'Jogos - Grupos'!$F$3:$F$74)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" s="116">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="H18" s="24">
         <f t="shared" si="1"/>
@@ -15246,7 +15254,7 @@
       </c>
       <c r="I18" s="116">
         <f t="shared" si="2"/>
-        <v>200000464</v>
+        <v>198000464</v>
       </c>
       <c r="J18" s="24">
         <f>RANK(I18,$I$15:$I$18,0)</f>
@@ -16697,15 +16705,15 @@
       </c>
       <c r="B55" s="135" t="str">
         <f>IFERROR(INDEX($B$11:$B$14,MATCH(1,$J$11:$J$14,0)),"?")</f>
-        <v>Brasil</v>
+        <v>Escocia</v>
       </c>
       <c r="C55" s="135" t="str">
         <f>IFERROR(INDEX($B$11:$B$14,MATCH(2,$J$11:$J$14,0)),"?")</f>
-        <v>Marrocos</v>
+        <v>Brasil</v>
       </c>
       <c r="D55" s="135" t="str">
         <f>IFERROR(INDEX($B$11:$B$14,MATCH(3,$J$11:$J$14,0)),"?")</f>
-        <v>Escocia</v>
+        <v>Marrocos</v>
       </c>
       <c r="E55" s="135" t="str">
         <f>IFERROR(INDEX($B$11:$B$14,MATCH(4,$J$11:$J$14,0)),"?")</f>
@@ -16929,7 +16937,7 @@
       </c>
       <c r="D68" s="150">
         <f t="shared" ref="D68:D79" si="3">RANK(C68,$C$68:$C$79,0)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -16946,7 +16954,7 @@
       </c>
       <c r="D69" s="150">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -16955,15 +16963,15 @@
       </c>
       <c r="B70" s="149" t="str">
         <f>IFERROR(INDEX($B$11:$B$14,MATCH(3,$J$11:$J$14,0)),"?")</f>
-        <v>Escocia</v>
+        <v>Marrocos</v>
       </c>
       <c r="C70" s="149">
         <f>IFERROR(INDEX($I$11:$I$14,MATCH(3,$J$11:$J$14,0)),0)</f>
-        <v>200000473</v>
+        <v>1200001486</v>
       </c>
       <c r="D70" s="150">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -16976,11 +16984,11 @@
       </c>
       <c r="C71" s="149">
         <f>IFERROR(INDEX($I$15:$I$18,MATCH(3,$J$15:$J$18,0)),0)</f>
-        <v>200000464</v>
+        <v>198000464</v>
       </c>
       <c r="D71" s="150">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -16997,7 +17005,7 @@
       </c>
       <c r="D72" s="150">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -17014,7 +17022,7 @@
       </c>
       <c r="D73" s="150">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -17048,7 +17056,7 @@
       </c>
       <c r="D75" s="150">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -17099,7 +17107,7 @@
       </c>
       <c r="D78" s="150">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -17116,7 +17124,7 @@
       </c>
       <c r="D79" s="150">
         <f t="shared" si="3"/>
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81" spans="1:2">
@@ -17133,7 +17141,7 @@
       </c>
       <c r="B82" s="164" t="str">
         <f>IFERROR(INDEX($B$68:$B$79,MATCH(1,$D$68:$D$79,0)),"?")</f>
-        <v>Canada</v>
+        <v>Marrocos</v>
       </c>
     </row>
     <row r="83" spans="1:2">
@@ -17142,7 +17150,7 @@
       </c>
       <c r="B83" s="164" t="str">
         <f>IFERROR(INDEX($B$68:$B$79,MATCH(2,$D$68:$D$79,0)),"?")</f>
-        <v>Suecia</v>
+        <v>Canada</v>
       </c>
     </row>
     <row r="84" spans="1:2">
@@ -17151,7 +17159,7 @@
       </c>
       <c r="B84" s="164" t="str">
         <f>IFERROR(INDEX($B$68:$B$79,MATCH(3,$D$68:$D$79,0)),"?")</f>
-        <v>Escocia</v>
+        <v>Suecia</v>
       </c>
     </row>
     <row r="85" spans="1:2">
@@ -17178,7 +17186,7 @@
       </c>
       <c r="B87" s="164" t="str">
         <f>IFERROR(INDEX($B$68:$B$79,MATCH(6,$D$68:$D$79,0)),"?")</f>
-        <v>Turquia</v>
+        <v>Egito</v>
       </c>
     </row>
     <row r="88" spans="1:2">
@@ -17187,7 +17195,7 @@
       </c>
       <c r="B88" s="164" t="str">
         <f>IFERROR(INDEX($B$68:$B$79,MATCH(7,$D$68:$D$79,0)),"?")</f>
-        <v>?</v>
+        <v>Costa do Marfim</v>
       </c>
     </row>
     <row r="89" spans="1:2">
@@ -17196,7 +17204,7 @@
       </c>
       <c r="B89" s="164" t="str">
         <f>IFERROR(INDEX($B$68:$B$79,MATCH(8,$D$68:$D$79,0)),"?")</f>
-        <v>Costa do Marfim</v>
+        <v>Gana</v>
       </c>
     </row>
     <row r="92" spans="1:2">
@@ -17205,7 +17213,7 @@
       </c>
       <c r="B92" s="166" t="str">
         <f>IF(D68&lt;=8,"A","")&amp;IF(D69&lt;=8,"B","")&amp;IF(D70&lt;=8,"C","")&amp;IF(D71&lt;=8,"D","")&amp;IF(D72&lt;=8,"E","")&amp;IF(D73&lt;=8,"F","")&amp;IF(D74&lt;=8,"G","")&amp;IF(D75&lt;=8,"H","")&amp;IF(D76&lt;=8,"I","")&amp;IF(D77&lt;=8,"J","")&amp;IF(D78&lt;=8,"K","")&amp;IF(D79&lt;=8,"L","")</f>
-        <v>BCDEFGIJ</v>
+        <v>BCEFGIJL</v>
       </c>
     </row>
   </sheetData>
@@ -43748,7 +43756,7 @@
       </c>
       <c r="E5" s="175" t="str">
         <f>IFERROR(IFERROR(INDEX('Classif - Grupos'!$B$68:$B$79,MATCH(MID(IFERROR(VLOOKUP('Classif - Grupos'!B92,'T495'!$A$2:$I$496,5,FALSE),""),2,1),'Classif - Grupos'!$A$68:$A$79,0)),"Aguardando"),"Aguardando")</f>
-        <v>Turquia</v>
+        <v>Marrocos</v>
       </c>
       <c r="F5" s="249"/>
       <c r="G5" s="249"/>
@@ -43778,7 +43786,7 @@
       </c>
       <c r="E6" s="175" t="str">
         <f>IFERROR('Classif - Grupos'!C55,"Aguardando")</f>
-        <v>Marrocos</v>
+        <v>Brasil</v>
       </c>
       <c r="F6" s="249"/>
       <c r="G6" s="249"/>
@@ -43804,7 +43812,7 @@
       </c>
       <c r="D7" s="175" t="str">
         <f>IFERROR('Classif - Grupos'!B55,"Aguardando")</f>
-        <v>Brasil</v>
+        <v>Escocia</v>
       </c>
       <c r="E7" s="175" t="str">
         <f>IFERROR('Classif - Grupos'!C58,"Aguardando")</f>
@@ -43898,7 +43906,7 @@
       </c>
       <c r="E10" s="175" t="str">
         <f>IFERROR(IFERROR(INDEX('Classif - Grupos'!$B$68:$B$79,MATCH(MID(IFERROR(VLOOKUP('Classif - Grupos'!B92,'T495'!$A$2:$I$496,2,FALSE),""),2,1),'Classif - Grupos'!$A$68:$A$79,0)),"Aguardando"),"Aguardando")</f>
-        <v>Escocia</v>
+        <v>Costa do Marfim</v>
       </c>
       <c r="F10" s="249"/>
       <c r="G10" s="249"/>
@@ -44138,7 +44146,7 @@
       </c>
       <c r="E18" s="175" t="str">
         <f>IFERROR(IFERROR(INDEX('Classif - Grupos'!$B$68:$B$79,MATCH(MID(IFERROR(VLOOKUP('Classif - Grupos'!B92,'T495'!$A$2:$I$496,8,FALSE),""),2,1),'Classif - Grupos'!$A$68:$A$79,0)),"Aguardando"),"Aguardando")</f>
-        <v>Costa do Marfim</v>
+        <v>Gana</v>
       </c>
       <c r="F18" s="249"/>
       <c r="G18" s="249"/>

</xml_diff>